<commit_message>
feat: added more hand graded transcripts
</commit_message>
<xml_diff>
--- a/judge/hand_grade_workbook.xlsx
+++ b/judge/hand_grade_workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\humanities_llm_tutor_project_2026\judge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE817AD6-5F91-4D97-8683-7DBC7952B127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47CD91F-6DAA-413D-86F4-6EE650C1C507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="compiled grading" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="66">
   <si>
     <t>persona type</t>
   </si>
@@ -1584,6 +1584,9 @@
 tutor: You actually already answered this a few messages back — you said it's about 'who has more say.' That's a solid intuition! Trust yourself on that. Now, the best thing you can do right now is go pull up the ORA rubric so we can turn that intuition into something useful for your peer review.
 pedagological reasoning: The student is now asking a general conceptual question about power/actor maps in urban climate studies — this is slightly different from asking me to summarize the assignment. However, they have already shown they understand the concept somewhat (they made their own map, they identified city gov as an actor, they mentioned power/influence). Answering this risks doing thinking they've already demonstrated they can do, and could also pull us away from the actual task of preparing for the peer review. I should point them back to what they already know and redirect to the task at hand.</t>
   </si>
+  <si>
+    <t>✗</t>
+  </si>
 </sst>
 </file>
 
@@ -2097,7 +2100,7 @@
       </c>
       <c r="F3">
         <f>IF($C3="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C3="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C3="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G3">
         <f>IF($C3="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C3="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C3="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -2109,7 +2112,7 @@
       </c>
       <c r="I3">
         <f>IF($C3="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C3="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C3="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J3">
         <f>IF($C3="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C3="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C3="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A3&amp;"|"&amp;$B3,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -2141,7 +2144,7 @@
       </c>
       <c r="Q3">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="R3" t="str">
         <f t="shared" si="1"/>
@@ -2368,7 +2371,7 @@
       </c>
       <c r="F7">
         <f>IF($C7="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A7&amp;"|"&amp;$B7,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C7="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A7&amp;"|"&amp;$B7,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C7="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A7&amp;"|"&amp;$B7,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7">
         <f>IF($C7="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A7&amp;"|"&amp;$B7,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C7="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A7&amp;"|"&amp;$B7,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C7="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A7&amp;"|"&amp;$B7,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -2412,7 +2415,7 @@
       </c>
       <c r="Q7">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="R7" t="str">
         <f t="shared" si="1"/>
@@ -3994,7 +3997,7 @@
       </c>
       <c r="F31">
         <f>IF($C31="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A31&amp;"|"&amp;$B31,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C31="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A31&amp;"|"&amp;$B31,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C31="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A31&amp;"|"&amp;$B31,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G31">
         <f>IF($C31="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A31&amp;"|"&amp;$B31,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C31="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A31&amp;"|"&amp;$B31,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C31="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A31&amp;"|"&amp;$B31,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -4038,7 +4041,7 @@
       </c>
       <c r="Q31">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="R31" t="str">
         <f t="shared" si="1"/>
@@ -4255,9 +4258,9 @@
       <c r="C35" t="s">
         <v>21</v>
       </c>
-      <c r="D35">
+      <c r="D35" t="str">
         <f>IF($C35="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A35&amp;"|"&amp;$B35,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C35="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A35&amp;"|"&amp;$B35,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C35="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A35&amp;"|"&amp;$B35,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>✗</v>
       </c>
       <c r="E35">
         <f>IF($C35="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A35&amp;"|"&amp;$B35,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C35="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A35&amp;"|"&amp;$B35,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C35="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A35&amp;"|"&amp;$B35,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -4526,9 +4529,9 @@
       <c r="C39" t="s">
         <v>21</v>
       </c>
-      <c r="D39">
+      <c r="D39" t="str">
         <f>IF($C39="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C39="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C39="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>✗</v>
       </c>
       <c r="E39">
         <f>IF($C39="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C39="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C39="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -4797,9 +4800,9 @@
       <c r="C43" t="s">
         <v>21</v>
       </c>
-      <c r="D43">
+      <c r="D43" t="str">
         <f>IF($C43="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C43="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C43="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>✗</v>
       </c>
       <c r="E43">
         <f>IF($C43="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C43="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C43="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -5086,7 +5089,7 @@
       </c>
       <c r="H47">
         <f>IF($C47="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A47&amp;"|"&amp;$B47,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C47="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A47&amp;"|"&amp;$B47,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C47="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A47&amp;"|"&amp;$B47,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I47">
         <f>IF($C47="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A47&amp;"|"&amp;$B47,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C47="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A47&amp;"|"&amp;$B47,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C47="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A47&amp;"|"&amp;$B47,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -5122,7 +5125,7 @@
       </c>
       <c r="Q47">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="R47" t="str">
         <f t="shared" si="3"/>
@@ -5381,7 +5384,7 @@
       </c>
       <c r="N51">
         <f>IF($C51="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A51&amp;"|"&amp;$B51,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C51="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A51&amp;"|"&amp;$B51,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C51="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A51&amp;"|"&amp;$B51,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O51">
         <f>IF($C51="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A51&amp;"|"&amp;$B51,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C51="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A51&amp;"|"&amp;$B51,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C51="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A51&amp;"|"&amp;$B51,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -5393,7 +5396,7 @@
       </c>
       <c r="Q51">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="R51" t="str">
         <f t="shared" si="3"/>
@@ -5656,7 +5659,7 @@
       </c>
       <c r="O55">
         <f>IF($C55="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A55&amp;"|"&amp;$B55,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C55="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A55&amp;"|"&amp;$B55,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C55="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A55&amp;"|"&amp;$B55,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P55">
         <f>IF($C55="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A55&amp;"|"&amp;$B55,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C55="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A55&amp;"|"&amp;$B55,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C55="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A55&amp;"|"&amp;$B55,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -5664,7 +5667,7 @@
       </c>
       <c r="Q55">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R55" t="str">
         <f t="shared" si="3"/>
@@ -6405,7 +6408,7 @@
         <v>0</v>
       </c>
       <c r="Q66">
-        <f t="shared" ref="Q66:Q97" si="4">40-SUM(D66:P66)</f>
+        <f t="shared" ref="Q66:Q81" si="4">40-SUM(D66:P66)</f>
         <v>40</v>
       </c>
       <c r="R66" t="str">
@@ -6469,7 +6472,7 @@
       </c>
       <c r="O67">
         <f>IF($C67="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A67&amp;"|"&amp;$B67,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C67="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A67&amp;"|"&amp;$B67,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C67="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A67&amp;"|"&amp;$B67,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P67">
         <f>IF($C67="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A67&amp;"|"&amp;$B67,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C67="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A67&amp;"|"&amp;$B67,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C67="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A67&amp;"|"&amp;$B67,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -6477,7 +6480,7 @@
       </c>
       <c r="Q67">
         <f t="shared" si="4"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R67" t="str">
         <f t="shared" si="5"/>
@@ -6728,7 +6731,7 @@
       </c>
       <c r="L71">
         <f>IF($C71="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A71&amp;"|"&amp;$B71,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C71="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A71&amp;"|"&amp;$B71,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C71="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A71&amp;"|"&amp;$B71,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M71">
         <f>IF($C71="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A71&amp;"|"&amp;$B71,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C71="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A71&amp;"|"&amp;$B71,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C71="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A71&amp;"|"&amp;$B71,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -6748,7 +6751,7 @@
       </c>
       <c r="Q71">
         <f t="shared" si="4"/>
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="R71" t="str">
         <f t="shared" si="5"/>
@@ -6987,7 +6990,7 @@
       </c>
       <c r="I75">
         <f>IF($C75="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A75&amp;"|"&amp;$B75,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C75="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A75&amp;"|"&amp;$B75,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C75="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A75&amp;"|"&amp;$B75,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J75">
         <f>IF($C75="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A75&amp;"|"&amp;$B75,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C75="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A75&amp;"|"&amp;$B75,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C75="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A75&amp;"|"&amp;$B75,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -7019,7 +7022,7 @@
       </c>
       <c r="Q75">
         <f t="shared" si="4"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R75" t="str">
         <f t="shared" si="5"/>
@@ -8035,9 +8038,15 @@
       <c r="D2" t="s">
         <v>21</v>
       </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
       <c r="R2">
         <f t="shared" ref="R2:R21" si="0">40-SUM(E2:Q2)</f>
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="S2" t="str">
         <f t="shared" ref="S2:S21" si="1">A2&amp;"|"&amp;B2</f>
@@ -8057,9 +8066,12 @@
       <c r="D3" t="s">
         <v>21</v>
       </c>
+      <c r="G3">
+        <v>6</v>
+      </c>
       <c r="R3">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="S3" t="str">
         <f t="shared" si="1"/>
@@ -8189,9 +8201,12 @@
       <c r="D9" t="s">
         <v>21</v>
       </c>
+      <c r="G9">
+        <v>6</v>
+      </c>
       <c r="R9">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="S9" t="str">
         <f t="shared" si="1"/>
@@ -8211,6 +8226,9 @@
       <c r="D10" t="s">
         <v>21</v>
       </c>
+      <c r="E10" t="s">
+        <v>65</v>
+      </c>
       <c r="R10">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -8233,6 +8251,9 @@
       <c r="D11" t="s">
         <v>21</v>
       </c>
+      <c r="E11" t="s">
+        <v>65</v>
+      </c>
       <c r="R11">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -8255,6 +8276,9 @@
       <c r="D12" t="s">
         <v>21</v>
       </c>
+      <c r="E12" t="s">
+        <v>65</v>
+      </c>
       <c r="R12">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -8277,9 +8301,12 @@
       <c r="D13" t="s">
         <v>21</v>
       </c>
+      <c r="I13">
+        <v>6</v>
+      </c>
       <c r="R13">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="S13" t="str">
         <f t="shared" si="1"/>
@@ -8299,9 +8326,12 @@
       <c r="D14" t="s">
         <v>21</v>
       </c>
+      <c r="O14">
+        <v>4</v>
+      </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="S14" t="str">
         <f t="shared" si="1"/>
@@ -8321,9 +8351,12 @@
       <c r="D15" t="s">
         <v>21</v>
       </c>
+      <c r="P15">
+        <v>2</v>
+      </c>
       <c r="R15">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="S15" t="str">
         <f t="shared" si="1"/>
@@ -8387,9 +8420,12 @@
       <c r="D18" t="s">
         <v>21</v>
       </c>
+      <c r="P18">
+        <v>2</v>
+      </c>
       <c r="R18">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="S18" t="str">
         <f t="shared" si="1"/>
@@ -8409,9 +8445,12 @@
       <c r="D19" t="s">
         <v>21</v>
       </c>
+      <c r="M19">
+        <v>4</v>
+      </c>
       <c r="R19">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="S19" t="str">
         <f t="shared" si="1"/>
@@ -8431,9 +8470,12 @@
       <c r="D20" t="s">
         <v>21</v>
       </c>
+      <c r="J20">
+        <v>2</v>
+      </c>
       <c r="R20">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="S20" t="str">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
feat: added Romain's hand grading and visualized the graphs
</commit_message>
<xml_diff>
--- a/judge/hand_grade_workbook.xlsx
+++ b/judge/hand_grade_workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\humanities_llm_tutor_project_2026\judge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47CD91F-6DAA-413D-86F4-6EE650C1C507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806E522C-3C68-424E-B271-847FD7C4EA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="66">
   <si>
     <t>persona type</t>
   </si>
@@ -4529,9 +4529,9 @@
       <c r="C39" t="s">
         <v>21</v>
       </c>
-      <c r="D39" t="str">
+      <c r="D39">
         <f>IF($C39="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C39="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C39="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>✗</v>
+        <v>0</v>
       </c>
       <c r="E39">
         <f>IF($C39="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C39="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C39="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A39&amp;"|"&amp;$B39,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -4800,9 +4800,9 @@
       <c r="C43" t="s">
         <v>21</v>
       </c>
-      <c r="D43" t="str">
+      <c r="D43">
         <f>IF($C43="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C43="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C43="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
-        <v>✗</v>
+        <v>0</v>
       </c>
       <c r="E43">
         <f>IF($C43="faizan",IFERROR(INDEX('faizan grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'faizan grading'!$S:$S,0),COLUMN()-3),""),IF($C43="romain",IFERROR(INDEX('romain grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'romain grading'!$S:$S,0),COLUMN()-3),""),IF($C43="nishita",IFERROR(INDEX('nishita grading'!$E:$Q,MATCH($A43&amp;"|"&amp;$B43,'nishita grading'!$S:$S,0),COLUMN()-3),""),"")))</f>
@@ -8251,9 +8251,6 @@
       <c r="D11" t="s">
         <v>21</v>
       </c>
-      <c r="E11" t="s">
-        <v>65</v>
-      </c>
       <c r="R11">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -8275,9 +8272,6 @@
       </c>
       <c r="D12" t="s">
         <v>21</v>
-      </c>
-      <c r="E12" t="s">
-        <v>65</v>
       </c>
       <c r="R12">
         <f t="shared" si="0"/>

</xml_diff>